<commit_message>
docs: add style-preservation sample guidance
</commit_message>
<xml_diff>
--- a/samples/repeated_blocks_output.xlsx
+++ b/samples/repeated_blocks_output.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Styled table" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="One-cell list" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Empty repeat" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Directive-only styles" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -52,7 +53,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -79,6 +80,11 @@
         <fgColor rgb="FFE2F0D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -150,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -180,6 +186,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -796,4 +805,91 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Directive-only cells remain formatted blanks</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="3" t="n"/>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>The opening and closing tag cells keep their authored white fill and borders.</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="n"/>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>One</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="n"/>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Two</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="n"/>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Three</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n"/>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>Four</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Footer moves below all four fully formatted rows</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>